<commit_message>
Final few changes to project report before submitting. fixed negatives in the dataset that shouldnt be there.
</commit_message>
<xml_diff>
--- a/Data/Table1_clean.xlsx
+++ b/Data/Table1_clean.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connorpiercy/Documents/GitHub/Group_8_Project/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F70BD5-6EE5-B049-BCE3-A8E1ECBCA2D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{160A7E84-AB10-B94C-B945-7A7F6D6C8E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13980" yWindow="600" windowWidth="14820" windowHeight="16660" xr2:uid="{D913AFE5-FFEF-D343-BAB9-A12C62385E55}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{D913AFE5-FFEF-D343-BAB9-A12C62385E55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,6 +41,126 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
   <si>
+    <t>Jiu1_1</t>
+  </si>
+  <si>
+    <t>[0]</t>
+  </si>
+  <si>
+    <t>Tot1_1</t>
+  </si>
+  <si>
+    <t>Tot1_2</t>
+  </si>
+  <si>
+    <t>Tot1_3</t>
+  </si>
+  <si>
+    <t>Tez1_1</t>
+  </si>
+  <si>
+    <t>Tez1_2</t>
+  </si>
+  <si>
+    <t>Tez2_1</t>
+  </si>
+  <si>
+    <t>Tez2_2</t>
+  </si>
+  <si>
+    <t>Cua1_1</t>
+  </si>
+  <si>
+    <t>Cua1_2</t>
+  </si>
+  <si>
+    <t>Ca1_1</t>
+  </si>
+  <si>
+    <t>Ca1_2</t>
+  </si>
+  <si>
+    <t>CA2_1</t>
+  </si>
+  <si>
+    <t>CA2_2</t>
+  </si>
+  <si>
+    <t>CA2_3</t>
+  </si>
+  <si>
+    <t>[230]</t>
+  </si>
+  <si>
+    <t>CA2_4</t>
+  </si>
+  <si>
+    <t>[270]</t>
+  </si>
+  <si>
+    <t>CA3_1</t>
+  </si>
+  <si>
+    <t>CA3_2</t>
+  </si>
+  <si>
+    <t>Ca4_1</t>
+  </si>
+  <si>
+    <t>Ca4_2</t>
+  </si>
+  <si>
+    <t>Cec1_1</t>
+  </si>
+  <si>
+    <t>Cec1_2</t>
+  </si>
+  <si>
+    <t>Cec1_3</t>
+  </si>
+  <si>
+    <t>Cec1_4</t>
+  </si>
+  <si>
+    <t>Cec2_1</t>
+  </si>
+  <si>
+    <t>Cec2_2</t>
+  </si>
+  <si>
+    <t>TAM1_1</t>
+  </si>
+  <si>
+    <t>TAM1_2</t>
+  </si>
+  <si>
+    <t>[0.01]</t>
+  </si>
+  <si>
+    <t>TAJ1_1</t>
+  </si>
+  <si>
+    <t>TAJ1_2</t>
+  </si>
+  <si>
+    <t>TAJ1_3</t>
+  </si>
+  <si>
+    <t>TAJ1_4</t>
+  </si>
+  <si>
+    <t>TAC1_1</t>
+  </si>
+  <si>
+    <t>[0.00]</t>
+  </si>
+  <si>
+    <t>Elements</t>
+  </si>
+  <si>
+    <t>82-Pb</t>
+  </si>
+  <si>
     <t>11-Na*</t>
   </si>
   <si>
@@ -87,126 +207,6 @@
   </si>
   <si>
     <t>38-Sr</t>
-  </si>
-  <si>
-    <t>82-Pb</t>
-  </si>
-  <si>
-    <t>Jiu1_1</t>
-  </si>
-  <si>
-    <t>[0]</t>
-  </si>
-  <si>
-    <t>Tot1_1</t>
-  </si>
-  <si>
-    <t>Tot1_2</t>
-  </si>
-  <si>
-    <t>Tot1_3</t>
-  </si>
-  <si>
-    <t>Tez1_1</t>
-  </si>
-  <si>
-    <t>Tez1_2</t>
-  </si>
-  <si>
-    <t>Tez2_1</t>
-  </si>
-  <si>
-    <t>Tez2_2</t>
-  </si>
-  <si>
-    <t>Cua1_1</t>
-  </si>
-  <si>
-    <t>Cua1_2</t>
-  </si>
-  <si>
-    <t>Ca1_1</t>
-  </si>
-  <si>
-    <t>Ca1_2</t>
-  </si>
-  <si>
-    <t>CA2_1</t>
-  </si>
-  <si>
-    <t>CA2_2</t>
-  </si>
-  <si>
-    <t>CA2_3</t>
-  </si>
-  <si>
-    <t>[230]</t>
-  </si>
-  <si>
-    <t>CA2_4</t>
-  </si>
-  <si>
-    <t>[270]</t>
-  </si>
-  <si>
-    <t>CA3_1</t>
-  </si>
-  <si>
-    <t>CA3_2</t>
-  </si>
-  <si>
-    <t>Ca4_1</t>
-  </si>
-  <si>
-    <t>Ca4_2</t>
-  </si>
-  <si>
-    <t>Cec1_1</t>
-  </si>
-  <si>
-    <t>Cec1_2</t>
-  </si>
-  <si>
-    <t>Cec1_3</t>
-  </si>
-  <si>
-    <t>Cec1_4</t>
-  </si>
-  <si>
-    <t>Cec2_1</t>
-  </si>
-  <si>
-    <t>Cec2_2</t>
-  </si>
-  <si>
-    <t>TAM1_1</t>
-  </si>
-  <si>
-    <t>TAM1_2</t>
-  </si>
-  <si>
-    <t>[0.01]</t>
-  </si>
-  <si>
-    <t>TAJ1_1</t>
-  </si>
-  <si>
-    <t>TAJ1_2</t>
-  </si>
-  <si>
-    <t>TAJ1_3</t>
-  </si>
-  <si>
-    <t>TAJ1_4</t>
-  </si>
-  <si>
-    <t>TAC1_1</t>
-  </si>
-  <si>
-    <t>[0.00]</t>
-  </si>
-  <si>
-    <t>Elements</t>
   </si>
 </sst>
 </file>
@@ -593,63 +593,63 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" t="s">
+        <v>51</v>
+      </c>
+      <c r="N1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q1" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>15</v>
-      </c>
       <c r="R1" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="B2">
         <v>0.28999999999999998</v>
@@ -685,10 +685,10 @@
         <v>620</v>
       </c>
       <c r="M2">
-        <v>-120</v>
+        <v>120</v>
       </c>
       <c r="N2">
-        <v>-15</v>
+        <v>15</v>
       </c>
       <c r="O2">
         <v>40</v>
@@ -705,7 +705,7 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>0.84</v>
@@ -741,10 +741,10 @@
         <v>840</v>
       </c>
       <c r="M3">
-        <v>-170</v>
+        <v>170</v>
       </c>
       <c r="N3">
-        <v>-14</v>
+        <v>14</v>
       </c>
       <c r="O3">
         <v>27</v>
@@ -761,7 +761,7 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0.2</v>
@@ -791,19 +791,19 @@
         <v>0.39</v>
       </c>
       <c r="K4">
-        <v>-1200</v>
+        <v>1200</v>
       </c>
       <c r="L4">
         <v>810</v>
       </c>
       <c r="M4">
-        <v>-130</v>
+        <v>130</v>
       </c>
       <c r="N4">
-        <v>-11</v>
+        <v>11</v>
       </c>
       <c r="O4">
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="P4">
         <v>21</v>
@@ -817,7 +817,7 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>0.45</v>
@@ -873,7 +873,7 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>0.28999999999999998</v>
@@ -903,22 +903,22 @@
         <v>0.38</v>
       </c>
       <c r="K6" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L6">
         <v>540</v>
       </c>
       <c r="M6">
-        <v>-270</v>
+        <v>270</v>
       </c>
       <c r="N6">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="O6">
-        <v>-8</v>
+        <v>8</v>
       </c>
       <c r="P6">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="Q6">
         <v>1430</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>0.32</v>
@@ -959,19 +959,19 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="K7" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L7">
         <v>660</v>
       </c>
       <c r="M7">
-        <v>-310</v>
+        <v>310</v>
       </c>
       <c r="N7">
-        <v>-6</v>
+        <v>6</v>
       </c>
       <c r="O7">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="P7">
         <v>15</v>
@@ -985,7 +985,7 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>1.26</v>
@@ -1015,22 +1015,22 @@
         <v>0.39</v>
       </c>
       <c r="K8" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L8">
         <v>600</v>
       </c>
       <c r="M8">
-        <v>-190</v>
+        <v>190</v>
       </c>
       <c r="N8">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="O8">
         <v>19</v>
       </c>
       <c r="P8">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="Q8">
         <v>900</v>
@@ -1041,7 +1041,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>1.71</v>
@@ -1071,16 +1071,16 @@
         <v>0.5</v>
       </c>
       <c r="K9" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L9">
-        <v>-520</v>
+        <v>520</v>
       </c>
       <c r="M9">
         <v>310</v>
       </c>
       <c r="N9">
-        <v>-14</v>
+        <v>14</v>
       </c>
       <c r="O9">
         <v>31</v>
@@ -1097,7 +1097,7 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>0.36</v>
@@ -1115,7 +1115,7 @@
         <v>0.22</v>
       </c>
       <c r="G10">
-        <v>-0.03</v>
+        <v>0.03</v>
       </c>
       <c r="H10">
         <v>0.14000000000000001</v>
@@ -1127,7 +1127,7 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="K10" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L10">
         <v>810</v>
@@ -1139,10 +1139,10 @@
         <v>25</v>
       </c>
       <c r="O10">
-        <v>-14</v>
+        <v>14</v>
       </c>
       <c r="P10">
-        <v>-14</v>
+        <v>14</v>
       </c>
       <c r="Q10">
         <v>8580</v>
@@ -1153,7 +1153,7 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>0.36</v>
@@ -1171,7 +1171,7 @@
         <v>0.18</v>
       </c>
       <c r="G11">
-        <v>-0.02</v>
+        <v>0.02</v>
       </c>
       <c r="H11">
         <v>0.12</v>
@@ -1183,7 +1183,7 @@
         <v>0.51</v>
       </c>
       <c r="K11" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L11">
         <v>820</v>
@@ -1195,7 +1195,7 @@
         <v>20</v>
       </c>
       <c r="O11">
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="P11">
         <v>14</v>
@@ -1209,7 +1209,7 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>0.3</v>
@@ -1239,7 +1239,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="K12">
-        <v>-170</v>
+        <v>170</v>
       </c>
       <c r="L12">
         <v>2070</v>
@@ -1265,7 +1265,7 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>0.15</v>
@@ -1295,7 +1295,7 @@
         <v>1.41</v>
       </c>
       <c r="K13" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L13">
         <v>1980</v>
@@ -1307,7 +1307,7 @@
         <v>32</v>
       </c>
       <c r="O13">
-        <v>-6</v>
+        <v>6</v>
       </c>
       <c r="P13">
         <v>34</v>
@@ -1321,7 +1321,7 @@
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>0.51</v>
@@ -1351,7 +1351,7 @@
         <v>0.99</v>
       </c>
       <c r="K14" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L14">
         <v>1330</v>
@@ -1363,7 +1363,7 @@
         <v>23</v>
       </c>
       <c r="O14">
-        <v>-4</v>
+        <v>4</v>
       </c>
       <c r="P14">
         <v>69</v>
@@ -1377,7 +1377,7 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>0.64</v>
@@ -1395,7 +1395,7 @@
         <v>0.66</v>
       </c>
       <c r="G15">
-        <v>-7.0000000000000007E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H15">
         <v>0.59</v>
@@ -1407,7 +1407,7 @@
         <v>1.74</v>
       </c>
       <c r="K15">
-        <v>-430</v>
+        <v>430</v>
       </c>
       <c r="L15">
         <v>2340</v>
@@ -1419,7 +1419,7 @@
         <v>17</v>
       </c>
       <c r="O15">
-        <v>-6</v>
+        <v>6</v>
       </c>
       <c r="P15">
         <v>16</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="B16">
-        <v>-0.28999999999999998</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="C16">
         <v>3.19</v>
@@ -1451,7 +1451,7 @@
         <v>0.43</v>
       </c>
       <c r="G16">
-        <v>-7.0000000000000007E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H16">
         <v>0.32</v>
@@ -1463,19 +1463,19 @@
         <v>0.75</v>
       </c>
       <c r="K16" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="L16">
         <v>2340</v>
       </c>
       <c r="M16">
-        <v>-260</v>
+        <v>260</v>
       </c>
       <c r="N16">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="O16">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="P16">
         <v>8</v>
@@ -1489,7 +1489,7 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B17">
         <v>0.44</v>
@@ -1507,7 +1507,7 @@
         <v>0.47</v>
       </c>
       <c r="G17">
-        <v>-0.05</v>
+        <v>0.05</v>
       </c>
       <c r="H17">
         <v>0.39</v>
@@ -1519,19 +1519,19 @@
         <v>0.76</v>
       </c>
       <c r="K17" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="L17">
         <v>2310</v>
       </c>
       <c r="M17">
-        <v>-150</v>
+        <v>150</v>
       </c>
       <c r="N17">
         <v>14</v>
       </c>
       <c r="O17">
-        <v>-5</v>
+        <v>5</v>
       </c>
       <c r="P17">
         <v>14</v>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="B18">
         <v>0.49</v>
@@ -1575,19 +1575,19 @@
         <v>0.93</v>
       </c>
       <c r="K18">
-        <v>-1300</v>
+        <v>1300</v>
       </c>
       <c r="L18">
         <v>2140</v>
       </c>
       <c r="M18">
-        <v>-360</v>
+        <v>360</v>
       </c>
       <c r="N18">
         <v>16</v>
       </c>
       <c r="O18">
-        <v>-4</v>
+        <v>4</v>
       </c>
       <c r="P18">
         <v>14</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B19">
         <v>0.7</v>
@@ -1619,7 +1619,7 @@
         <v>1</v>
       </c>
       <c r="G19">
-        <v>-7.0000000000000007E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H19">
         <v>0.6</v>
@@ -1631,19 +1631,19 @@
         <v>0.97</v>
       </c>
       <c r="K19">
-        <v>-1700</v>
+        <v>1700</v>
       </c>
       <c r="L19">
         <v>4560</v>
       </c>
       <c r="M19">
-        <v>-320</v>
+        <v>320</v>
       </c>
       <c r="N19">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="O19">
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="P19">
         <v>23</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="B20">
         <v>0.28999999999999998</v>
@@ -1687,7 +1687,7 @@
         <v>0.79</v>
       </c>
       <c r="K20">
-        <v>-940</v>
+        <v>940</v>
       </c>
       <c r="L20">
         <v>4580</v>
@@ -1699,7 +1699,7 @@
         <v>22</v>
       </c>
       <c r="O20">
-        <v>-7</v>
+        <v>7</v>
       </c>
       <c r="P20">
         <v>25</v>
@@ -1713,7 +1713,7 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="B21">
         <v>0.33</v>
@@ -1743,7 +1743,7 @@
         <v>0.78</v>
       </c>
       <c r="K21">
-        <v>-1260</v>
+        <v>1260</v>
       </c>
       <c r="L21">
         <v>3300</v>
@@ -1755,7 +1755,7 @@
         <v>18</v>
       </c>
       <c r="O21">
-        <v>-11</v>
+        <v>11</v>
       </c>
       <c r="P21">
         <v>26</v>
@@ -1769,7 +1769,7 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="B22">
         <v>0.23</v>
@@ -1799,7 +1799,7 @@
         <v>2.27</v>
       </c>
       <c r="K22" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L22">
         <v>2110</v>
@@ -1811,7 +1811,7 @@
         <v>30</v>
       </c>
       <c r="O22">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="P22">
         <v>60</v>
@@ -1825,7 +1825,7 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="B23">
         <v>0.11</v>
@@ -1855,7 +1855,7 @@
         <v>1.54</v>
       </c>
       <c r="K23" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L23">
         <v>1820</v>
@@ -1881,7 +1881,7 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B24">
         <v>0.56000000000000005</v>
@@ -1911,7 +1911,7 @@
         <v>1.32</v>
       </c>
       <c r="K24" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L24">
         <v>1320</v>
@@ -1937,7 +1937,7 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B25">
         <v>0.22</v>
@@ -1967,7 +1967,7 @@
         <v>1.54</v>
       </c>
       <c r="K25" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L25">
         <v>1870</v>
@@ -1993,7 +1993,7 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="B26">
         <v>0.2</v>
@@ -2023,7 +2023,7 @@
         <v>1.67</v>
       </c>
       <c r="K26" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L26">
         <v>1600</v>
@@ -2049,7 +2049,7 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="B27">
         <v>0.14000000000000001</v>
@@ -2079,7 +2079,7 @@
         <v>2.2200000000000002</v>
       </c>
       <c r="K27" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L27">
         <v>3880</v>
@@ -2105,10 +2105,10 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B28">
-        <v>-0.28999999999999998</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="C28">
         <v>2.25</v>
@@ -2123,7 +2123,7 @@
         <v>0.15</v>
       </c>
       <c r="G28">
-        <v>-0.02</v>
+        <v>0.02</v>
       </c>
       <c r="H28">
         <v>0.26</v>
@@ -2135,19 +2135,19 @@
         <v>1.49</v>
       </c>
       <c r="K28">
-        <v>-850</v>
+        <v>850</v>
       </c>
       <c r="L28">
         <v>1370</v>
       </c>
       <c r="M28">
-        <v>-250</v>
+        <v>250</v>
       </c>
       <c r="N28">
         <v>15</v>
       </c>
       <c r="O28">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="P28">
         <v>12</v>
@@ -2161,10 +2161,10 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B29">
-        <v>-0.19</v>
+        <v>0.19</v>
       </c>
       <c r="C29">
         <v>1.35</v>
@@ -2179,7 +2179,7 @@
         <v>0.22</v>
       </c>
       <c r="G29" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="H29">
         <v>0.2</v>
@@ -2191,22 +2191,22 @@
         <v>1.19</v>
       </c>
       <c r="K29">
-        <v>-850</v>
+        <v>850</v>
       </c>
       <c r="L29">
         <v>1040</v>
       </c>
       <c r="M29">
-        <v>-150</v>
+        <v>150</v>
       </c>
       <c r="N29">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="O29">
-        <v>-5</v>
+        <v>5</v>
       </c>
       <c r="P29">
-        <v>-8</v>
+        <v>8</v>
       </c>
       <c r="Q29">
         <v>300</v>
@@ -2217,7 +2217,7 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B30">
         <v>1.49</v>
@@ -2232,10 +2232,10 @@
         <v>16.5</v>
       </c>
       <c r="F30">
-        <v>-0.16</v>
+        <v>0.16</v>
       </c>
       <c r="G30">
-        <v>-7.0000000000000007E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H30">
         <v>0.43</v>
@@ -2247,19 +2247,19 @@
         <v>1.38</v>
       </c>
       <c r="K30" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L30">
         <v>1040</v>
       </c>
       <c r="M30">
-        <v>-280</v>
+        <v>280</v>
       </c>
       <c r="N30">
         <v>22</v>
       </c>
       <c r="O30" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="P30">
         <v>15</v>
@@ -2273,10 +2273,10 @@
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B31">
-        <v>-0.2</v>
+        <v>0.2</v>
       </c>
       <c r="C31">
         <v>1.26</v>
@@ -2291,10 +2291,10 @@
         <v>0.1</v>
       </c>
       <c r="G31" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="H31">
-        <v>-0.06</v>
+        <v>0.06</v>
       </c>
       <c r="I31">
         <v>53.1</v>
@@ -2303,19 +2303,19 @@
         <v>0.54</v>
       </c>
       <c r="K31">
-        <v>-1530</v>
+        <v>1530</v>
       </c>
       <c r="L31">
         <v>850</v>
       </c>
       <c r="M31">
-        <v>-170</v>
+        <v>170</v>
       </c>
       <c r="N31">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="O31">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="P31">
         <v>10</v>
@@ -2329,10 +2329,10 @@
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="B32">
-        <v>-0.19</v>
+        <v>0.19</v>
       </c>
       <c r="C32">
         <v>3.37</v>
@@ -2344,10 +2344,10 @@
         <v>17.899999999999999</v>
       </c>
       <c r="F32">
-        <v>-0.06</v>
+        <v>0.06</v>
       </c>
       <c r="G32">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="H32">
         <v>0.27</v>
@@ -2359,19 +2359,19 @@
         <v>0.76</v>
       </c>
       <c r="K32">
-        <v>-590</v>
+        <v>590</v>
       </c>
       <c r="L32">
         <v>1470</v>
       </c>
       <c r="M32">
-        <v>-140</v>
+        <v>140</v>
       </c>
       <c r="N32">
         <v>12</v>
       </c>
       <c r="O32">
-        <v>-5</v>
+        <v>5</v>
       </c>
       <c r="P32">
         <v>8</v>
@@ -2385,10 +2385,10 @@
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="B33">
-        <v>-0.43</v>
+        <v>0.43</v>
       </c>
       <c r="C33">
         <v>0.38</v>
@@ -2400,7 +2400,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="F33">
-        <v>-0.09</v>
+        <v>0.09</v>
       </c>
       <c r="G33">
         <v>0.22</v>
@@ -2415,19 +2415,19 @@
         <v>1.18</v>
       </c>
       <c r="K33">
-        <v>-690</v>
+        <v>690</v>
       </c>
       <c r="L33">
         <v>1600</v>
       </c>
       <c r="M33">
-        <v>-240</v>
+        <v>240</v>
       </c>
       <c r="N33">
-        <v>-29</v>
+        <v>29</v>
       </c>
       <c r="O33">
-        <v>-17</v>
+        <v>17</v>
       </c>
       <c r="P33">
         <v>21</v>
@@ -2441,7 +2441,7 @@
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B34">
         <v>0.56000000000000005</v>
@@ -2459,7 +2459,7 @@
         <v>0.36</v>
       </c>
       <c r="G34">
-        <v>-0.02</v>
+        <v>0.02</v>
       </c>
       <c r="H34">
         <v>0.9</v>
@@ -2471,7 +2471,7 @@
         <v>5.18</v>
       </c>
       <c r="K34">
-        <v>-1000</v>
+        <v>1000</v>
       </c>
       <c r="L34">
         <v>3920</v>
@@ -2483,7 +2483,7 @@
         <v>154</v>
       </c>
       <c r="O34">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="P34">
         <v>52</v>
@@ -2497,7 +2497,7 @@
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B35">
         <v>0.4</v>
@@ -2515,7 +2515,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G35" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="H35">
         <v>0.14000000000000001</v>
@@ -2527,19 +2527,19 @@
         <v>0.86</v>
       </c>
       <c r="K35">
-        <v>-1320</v>
+        <v>1320</v>
       </c>
       <c r="L35">
         <v>1310</v>
       </c>
       <c r="M35">
-        <v>-250</v>
+        <v>250</v>
       </c>
       <c r="N35">
-        <v>-11</v>
+        <v>11</v>
       </c>
       <c r="O35">
-        <v>-4</v>
+        <v>4</v>
       </c>
       <c r="P35">
         <v>12</v>
@@ -2553,7 +2553,7 @@
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B36">
         <v>0.41</v>
@@ -2571,7 +2571,7 @@
         <v>0.16</v>
       </c>
       <c r="G36">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="H36">
         <v>0.14000000000000001</v>
@@ -2583,22 +2583,22 @@
         <v>0.61</v>
       </c>
       <c r="K36">
-        <v>-1340</v>
+        <v>1340</v>
       </c>
       <c r="L36">
         <v>1250</v>
       </c>
       <c r="M36">
-        <v>-200</v>
+        <v>200</v>
       </c>
       <c r="N36">
-        <v>-14</v>
+        <v>14</v>
       </c>
       <c r="O36">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="P36">
-        <v>-6</v>
+        <v>6</v>
       </c>
       <c r="Q36">
         <v>340</v>

</xml_diff>